<commit_message>
Add auditable cash-flow workbench and filing-backed diligence
</commit_message>
<xml_diff>
--- a/finance/downloads/industrial-investment-model.xlsx
+++ b/finance/downloads/industrial-investment-model.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra26af2fa23e4490b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rab8107d996ec4047"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R1f189d75cb7f4d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="4" r:id="R83056c128c1f48f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="5" r:id="R6979a1cd853c498d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="6" r:id="Rb85bb740d6ac476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Screen" sheetId="7" r:id="R3271aaaca30d4ede"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="8" r:id="R6a06bdf1c5c24237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R13312497dbf946ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R0b8b89fbf58343e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R2a59721b398a4c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="4" r:id="R49c8552a53704b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="5" r:id="R0c509c3e00554a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="6" r:id="Redf9a12934dc41a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Screen" sheetId="7" r:id="R625dd686e38c472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="8" r:id="Rebbc37977c3546cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -981,7 +981,7 @@
       <x:c r="D17" s="3"/>
       <x:c r="E17" s="56" t="n">
         <x:f>'Valuation'!E51</x:f>
-        <x:v>1076.0506348383283</x:v>
+        <x:v>892.5856406199086</x:v>
       </x:c>
       <x:c r="F17" s="3"/>
       <x:c r="G17" s="3"/>
@@ -3552,9 +3552,13 @@
     <x:row r="58" ht="20" customHeight="1">
       <x:c r="A58" s="2"/>
       <x:c r="B58" s="2"/>
-      <x:c r="C58" s="2"/>
+      <x:c r="C58" s="2" t="str">
+        <x:v>Terminal return on invested capital</x:v>
+      </x:c>
       <x:c r="D58" s="3"/>
-      <x:c r="E58" s="3"/>
+      <x:c r="E58" s="30" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
       <x:c r="F58" s="3"/>
       <x:c r="G58" s="3"/>
       <x:c r="H58" s="3"/>
@@ -4678,7 +4682,7 @@
       <x:c r="A21" s="2"/>
       <x:c r="B21" s="2"/>
       <x:c r="C21" s="28" t="str">
-        <x:v>Free cash flow before debt service</x:v>
+        <x:v>Levered FCF before principal payments</x:v>
       </x:c>
       <x:c r="D21" s="29"/>
       <x:c r="E21" s="29" t="n">
@@ -6141,7 +6145,7 @@
       <x:c r="A11" s="2"/>
       <x:c r="B11" s="2"/>
       <x:c r="C11" s="2" t="str">
-        <x:v>Free cash flow before debt service</x:v>
+        <x:v>Levered FCF before principal payments</x:v>
       </x:c>
       <x:c r="D11" s="3"/>
       <x:c r="E11" s="8" t="n">
@@ -7991,7 +7995,7 @@
       <x:c r="D15" s="3"/>
       <x:c r="E15" s="8" t="n">
         <x:f>E8-'Inputs'!E23+'Inputs'!E16</x:f>
-        <x:v>955.803</x:v>
+        <x:v>955.053</x:v>
       </x:c>
       <x:c r="F15" s="3"/>
       <x:c r="G15" s="3"/>
@@ -8014,7 +8018,7 @@
       <x:c r="D16" s="3"/>
       <x:c r="E16" s="8" t="n">
         <x:f>'Inputs'!E23</x:f>
-        <x:v>310</x:v>
+        <x:v>310.75</x:v>
       </x:c>
       <x:c r="F16" s="3"/>
       <x:c r="G16" s="3"/>
@@ -8651,12 +8655,12 @@
       <x:c r="A45" s="2"/>
       <x:c r="B45" s="2"/>
       <x:c r="C45" s="2" t="str">
-        <x:v>Terminal capex</x:v>
+        <x:v>Terminal NOPAT</x:v>
       </x:c>
       <x:c r="D45" s="3"/>
       <x:c r="E45" s="8" t="n">
-        <x:f>E42*'Assumptions'!E23</x:f>
-        <x:v>27.23156228323934</x:v>
+        <x:f>E43-E44-MAX(0,E43-E44)*'Assumptions'!E22</x:f>
+        <x:v>89.19319687489536</x:v>
       </x:c>
       <x:c r="F45" s="3"/>
       <x:c r="G45" s="3"/>
@@ -8674,12 +8678,12 @@
       <x:c r="A46" s="2"/>
       <x:c r="B46" s="2"/>
       <x:c r="C46" s="2" t="str">
-        <x:v>Terminal working-capital investment</x:v>
+        <x:v>Terminal reinvestment (growth / ROIC)</x:v>
       </x:c>
       <x:c r="D46" s="3"/>
       <x:c r="E46" s="8" t="n">
-        <x:f>'Forecast'!I19*E41</x:f>
-        <x:v>3.744979298877441</x:v>
+        <x:f>IF('Assumptions'!E58&gt;0,MAX(0,E45)*E41/'Assumptions'!E58,NA())</x:f>
+        <x:v>18.581916015603202</x:v>
       </x:c>
       <x:c r="F46" s="3"/>
       <x:c r="G46" s="3"/>
@@ -8700,9 +8704,9 @@
         <x:v>Terminal unlevered cash flow</x:v>
       </x:c>
       <x:c r="D47" s="3"/>
-      <x:c r="E47" s="8" t="n">
-        <x:f>E43-MAX(0,E43-E44)*'Assumptions'!E22-E45-E46</x:f>
-        <x:v>92.77169644719523</x:v>
+      <x:c r="E47" s="3" t="n">
+        <x:f>E45-E46</x:f>
+        <x:v>70.61128085929217</x:v>
       </x:c>
       <x:c r="F47" s="3"/>
       <x:c r="G47" s="3"/>
@@ -8725,7 +8729,7 @@
       <x:c r="D48" s="3"/>
       <x:c r="E48" s="3" t="n">
         <x:f>IF(E40&gt;E41,E47/(E40-E41),NA())</x:f>
-        <x:v>1236.9559526292694</x:v>
+        <x:v>941.483744790562</x:v>
       </x:c>
       <x:c r="F48" s="3"/>
       <x:c r="G48" s="3"/>
@@ -8771,7 +8775,7 @@
       <x:c r="D50" s="3"/>
       <x:c r="E50" s="3" t="n">
         <x:f>E48/(1+E40)^5</x:f>
-        <x:v>768.0523266724633</x:v>
+        <x:v>584.5873324540436</x:v>
       </x:c>
       <x:c r="F50" s="3"/>
       <x:c r="G50" s="3"/>
@@ -8794,7 +8798,7 @@
       <x:c r="D51" s="29"/>
       <x:c r="E51" s="29" t="n">
         <x:f>SUM(E49:E50)</x:f>
-        <x:v>1076.0506348383283</x:v>
+        <x:v>892.5856406199086</x:v>
       </x:c>
       <x:c r="F51" s="29"/>
       <x:c r="G51" s="29"/>
@@ -8817,7 +8821,7 @@
       <x:c r="D52" s="29"/>
       <x:c r="E52" s="49" t="n">
         <x:f>E51-'Inputs'!E23+'Inputs'!E16</x:f>
-        <x:v>801.1336348383282</x:v>
+        <x:v>616.9186406199086</x:v>
       </x:c>
       <x:c r="F52" s="29"/>
       <x:c r="G52" s="29"/>
@@ -8891,7 +8895,7 @@
       <x:c r="A56" s="2"/>
       <x:c r="B56" s="2"/>
       <x:c r="C56" s="21" t="str">
-        <x:v>DCF discount rate is assumed. Terminal working capital is recomputed at terminal growth.</x:v>
+        <x:v>DCF discount rate is assumed. Reinvestment = positive terminal NOPAT x growth / terminal ROIC.</x:v>
       </x:c>
       <x:c r="D56" s="22"/>
       <x:c r="E56" s="22"/>
@@ -11900,7 +11904,7 @@
       <x:c r="A30" s="2"/>
       <x:c r="B30" s="2"/>
       <x:c r="C30" s="2" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/42682/000119312526040888/grc-ex99.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/42682/000119312526084820/grc-20251231.htm</x:v>
       </x:c>
       <x:c r="D30" s="3"/>
       <x:c r="E30" s="3"/>
@@ -12842,7 +12846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cd6f89ee4af4161"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0811e24f6b764f9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13380,7 +13384,7 @@
       </x:c>
       <x:c r="D23" s="3"/>
       <x:c r="E23" s="20" t="n">
-        <x:v>310</x:v>
+        <x:v>310.75</x:v>
       </x:c>
       <x:c r="F23" s="3"/>
       <x:c r="G23" s="3"/>
@@ -13440,7 +13444,7 @@
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="2"/>
       <x:c r="C26" s="21" t="str">
-        <x:v>Source: Gorman-Rupp FY2025 earnings release, February 6, 2026.</x:v>
+        <x:v>Source: audited FY2025 10-K, March 2, 2026, pp.29-31.</x:v>
       </x:c>
       <x:c r="D26" s="22"/>
       <x:c r="E26" s="22"/>
@@ -13460,7 +13464,7 @@
       <x:c r="A27" s="2"/>
       <x:c r="B27" s="2"/>
       <x:c r="C27" s="23" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/42682/000119312526040888/grc-ex99.htm</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/42682/000119312526084820/grc-20251231.htm</x:v>
       </x:c>
       <x:c r="D27" s="3"/>
       <x:c r="E27" s="3"/>
@@ -13498,7 +13502,7 @@
       <x:c r="A29" s="2"/>
       <x:c r="B29" s="2"/>
       <x:c r="C29" s="21" t="str">
-        <x:v>The release’s condensed statements are unaudited. Data retrieved September 23, 2026.</x:v>
+        <x:v>Audited statements. Data checked September 23, 2026. Model version 2.</x:v>
       </x:c>
       <x:c r="D29" s="22"/>
       <x:c r="E29" s="22"/>
@@ -13558,7 +13562,7 @@
       <x:c r="A32" s="2"/>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="21" t="str">
-        <x:v>The model uses operating income + D&amp;A, not company-adjusted EBITDA.</x:v>
+        <x:v>Operating EBITDA uses operating income + D&amp;A; management adjustments are separate.</x:v>
       </x:c>
       <x:c r="D32" s="22"/>
       <x:c r="E32" s="22"/>
@@ -13595,7 +13599,9 @@
     <x:row r="34" ht="20" customHeight="1">
       <x:c r="A34" s="2"/>
       <x:c r="B34" s="2"/>
-      <x:c r="C34" s="2"/>
+      <x:c r="C34" s="2" t="str">
+        <x:v>Adjusted EBITDA source: FY2025 earnings reconciliation, February 6, 2026.</x:v>
+      </x:c>
       <x:c r="D34" s="3"/>
       <x:c r="E34" s="3"/>
       <x:c r="F34" s="3"/>
@@ -13613,7 +13619,9 @@
     <x:row r="35" ht="20" customHeight="1">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="2"/>
-      <x:c r="C35" s="2"/>
+      <x:c r="C35" s="2" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/42682/000119312526040888/grc-ex99.htm</x:v>
+      </x:c>
       <x:c r="D35" s="3"/>
       <x:c r="E35" s="3"/>
       <x:c r="F35" s="3"/>

</xml_diff>